<commit_message>
fix: review points on the reference cases (PLAN.md 3.4)
Case 23 grows, so it no longer claims to cover zero growth; the formula
guard also refuses a minus after any operator and chained powers (both read
differently in Excel); the index links to each sheet with HYPERLINK, which
every viewer follows. Verified: tests/test_reference_cases.py passes and the
guard refuses x * -y and a ** b ** c.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reference/reference_cases.xlsx
+++ b/tests/reference/reference_cases.xlsx
@@ -526,10 +526,9 @@
       <c r="D5" t="n">
         <v>44</v>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>01_no_leverage</t>
-        </is>
+      <c r="E5">
+        <f>HYPERLINK("#'01_no_leverage'!A1", "01_no_leverage")</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -549,10 +548,9 @@
       <c r="D6" t="n">
         <v>42</v>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>02_single_bullet</t>
-        </is>
+      <c r="E6">
+        <f>HYPERLINK("#'02_single_bullet'!A1", "02_single_bullet")</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -572,10 +570,9 @@
       <c r="D7" t="n">
         <v>51</v>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>03_single_sweep</t>
-        </is>
+      <c r="E7">
+        <f>HYPERLINK("#'03_single_sweep'!A1", "03_single_sweep")</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -595,10 +592,9 @@
       <c r="D8" t="n">
         <v>48</v>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>04_amortising</t>
-        </is>
+      <c r="E8">
+        <f>HYPERLINK("#'04_amortising'!A1", "04_amortising")</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -618,10 +614,9 @@
       <c r="D9" t="n">
         <v>42</v>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>05_fees_only</t>
-        </is>
+      <c r="E9">
+        <f>HYPERLINK("#'05_fees_only'!A1", "05_fees_only")</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -641,10 +636,9 @@
       <c r="D10" t="n">
         <v>42</v>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>06_fees_on_debt</t>
-        </is>
+      <c r="E10">
+        <f>HYPERLINK("#'06_fees_on_debt'!A1", "06_fees_on_debt")</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -664,10 +658,9 @@
       <c r="D11" t="n">
         <v>51</v>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>07_percentage_structure</t>
-        </is>
+      <c r="E11">
+        <f>HYPERLINK("#'07_percentage_structure'!A1", "07_percentage_structure")</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -687,10 +680,9 @@
       <c r="D12" t="n">
         <v>38</v>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>08_finding_11</t>
-        </is>
+      <c r="E12">
+        <f>HYPERLINK("#'08_finding_11'!A1", "08_finding_11")</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -710,10 +702,9 @@
       <c r="D13" t="n">
         <v>42</v>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>09_sonia_floor</t>
-        </is>
+      <c r="E13">
+        <f>HYPERLINK("#'09_sonia_floor'!A1", "09_sonia_floor")</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -733,10 +724,9 @@
       <c r="D14" t="n">
         <v>48</v>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>10_pik</t>
-        </is>
+      <c r="E14">
+        <f>HYPERLINK("#'10_pik'!A1", "10_pik")</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -756,10 +746,9 @@
       <c r="D15" t="n">
         <v>51</v>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>11_unitranche_half_sweep</t>
-        </is>
+      <c r="E15">
+        <f>HYPERLINK("#'11_unitranche_half_sweep'!A1", "11_unitranche_half_sweep")</f>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -779,10 +768,9 @@
       <c r="D16" t="n">
         <v>51</v>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>12_two_tranche_waterfall</t>
-        </is>
+      <c r="E16">
+        <f>HYPERLINK("#'12_two_tranche_waterfall'!A1", "12_two_tranche_waterfall")</f>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -802,10 +790,9 @@
       <c r="D17" t="n">
         <v>36</v>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>13_revolver</t>
-        </is>
+      <c r="E17">
+        <f>HYPERLINK("#'13_revolver'!A1", "13_revolver")</f>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -825,10 +812,9 @@
       <c r="D18" t="n">
         <v>45</v>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>14_interest_cap</t>
-        </is>
+      <c r="E18">
+        <f>HYPERLINK("#'14_interest_cap'!A1", "14_interest_cap")</f>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -848,10 +834,9 @@
       <c r="D19" t="n">
         <v>48</v>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>15_interest_cap_used</t>
-        </is>
+      <c r="E19">
+        <f>HYPERLINK("#'15_interest_cap_used'!A1", "15_interest_cap_used")</f>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -871,10 +856,9 @@
       <c r="D20" t="n">
         <v>51</v>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>16_tax_losses</t>
-        </is>
+      <c r="E20">
+        <f>HYPERLINK("#'16_tax_losses'!A1", "16_tax_losses")</f>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -894,10 +878,9 @@
       <c r="D21" t="n">
         <v>51</v>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>17_loss_limit</t>
-        </is>
+      <c r="E21">
+        <f>HYPERLINK("#'17_loss_limit'!A1", "17_loss_limit")</f>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -917,10 +900,9 @@
       <c r="D22" t="n">
         <v>45</v>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>18_minimum_tax</t>
-        </is>
+      <c r="E22">
+        <f>HYPERLINK("#'18_minimum_tax'!A1", "18_minimum_tax")</f>
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -940,10 +922,9 @@
       <c r="D23" t="n">
         <v>44</v>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>19_ifrs16_post</t>
-        </is>
+      <c r="E23">
+        <f>HYPERLINK("#'19_ifrs16_post'!A1", "19_ifrs16_post")</f>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -963,10 +944,9 @@
       <c r="D24" t="n">
         <v>42</v>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>20_ifrs16_pre</t>
-        </is>
+      <c r="E24">
+        <f>HYPERLINK("#'20_ifrs16_pre'!A1", "20_ifrs16_pre")</f>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -986,10 +966,9 @@
       <c r="D25" t="n">
         <v>42</v>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>21_euro_thousands</t>
-        </is>
+      <c r="E25">
+        <f>HYPERLINK("#'21_euro_thousands'!A1", "21_euro_thousands")</f>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -1009,10 +988,9 @@
       <c r="D26" t="n">
         <v>43</v>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>22_march_year_end_yen</t>
-        </is>
+      <c r="E26">
+        <f>HYPERLINK("#'22_march_year_end_yen'!A1", "22_march_year_end_yen")</f>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -1026,16 +1004,15 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>zero growth</t>
+          <t>single tranche</t>
         </is>
       </c>
       <c r="D27" t="n">
         <v>42</v>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>23_growth_working_capital_days</t>
-        </is>
+      <c r="E27">
+        <f>HYPERLINK("#'23_growth_working_capital_days'!A1", "23_growth_working_capital_days")</f>
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -1055,10 +1032,9 @@
       <c r="D28" t="n">
         <v>44</v>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>24_minimum_cash</t>
-        </is>
+      <c r="E28">
+        <f>HYPERLINK("#'24_minimum_cash'!A1", "24_minimum_cash")</f>
+        <v/>
       </c>
     </row>
     <row r="29">
@@ -1078,10 +1054,9 @@
       <c r="D29" t="n">
         <v>18</v>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>25_one_year_hold</t>
-        </is>
+      <c r="E29">
+        <f>HYPERLINK("#'25_one_year_hold'!A1", "25_one_year_hold")</f>
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -1101,44 +1076,15 @@
       <c r="D30" t="n">
         <v>54</v>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>26_shared_sweep</t>
-        </is>
+      <c r="E30">
+        <f>HYPERLINK("#'26_shared_sweep'!A1", "26_shared_sweep")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId26"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -28301,7 +28247,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Covers: zero growth</t>
+          <t>Covers: single tranche</t>
         </is>
       </c>
     </row>

</xml_diff>